<commit_message>
completed all bugs points
</commit_message>
<xml_diff>
--- a/Source/SmartInventory/SmartInventory/Content/Templates/Site/ImportSite.xlsx
+++ b/Source/SmartInventory/SmartInventory/Content/Templates/Site/ImportSite.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19035" windowHeight="7620"/>
+    <workbookView windowWidth="19635" windowHeight="7620"/>
   </bookViews>
   <sheets>
     <sheet name="Site" sheetId="1" r:id="rId1"/>
@@ -465,7 +465,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -486,28 +486,6 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -634,7 +612,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -646,34 +624,34 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -758,7 +736,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
@@ -780,10 +758,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -794,7 +769,7 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
@@ -1059,13 +1034,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
-<customStorage xmlns="https://web.wps.cn/et/2018/main">
-  <book/>
-  <sheets/>
-</customStorage>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1403,45 +1371,21 @@
         <v>15</v>
       </c>
       <c r="H2" s="5"/>
-      <c r="I2" s="7"/>
+      <c r="I2" s="5"/>
       <c r="J2" s="5" t="s">
         <v>16</v>
       </c>
       <c r="K2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:1">
       <c r="A3" s="6"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:1">
       <c r="A4" s="6"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="8"/>
-      <c r="M4" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>